<commit_message>
DMS Report module added
</commit_message>
<xml_diff>
--- a/_data_list/FF_RY.xlsx
+++ b/_data_list/FF_RY.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Telegram_Project\OrangeFlow_Dev\_data_list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAC4021C-F05D-449D-9DF0-05969114C625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65BE9C60-7E8B-428F-98DD-2552AAA29425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="130">
   <si>
     <t>DMS_CODE</t>
   </si>
@@ -417,6 +417,18 @@
   </si>
   <si>
     <t>Father</t>
+  </si>
+  <si>
+    <t>Chondiber</t>
+  </si>
+  <si>
+    <t>Rail Way High School</t>
+  </si>
+  <si>
+    <t>Bilkis Begum</t>
+  </si>
+  <si>
+    <t>Kalshi Mirpur, Pollobi, Dhaka uttor city corporation, Dhaka</t>
   </si>
 </sst>
 </file>
@@ -502,7 +514,27 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1064,6 +1096,9 @@
       <c r="D3" s="5" t="s">
         <v>37</v>
       </c>
+      <c r="F3" s="5">
+        <v>1410071973</v>
+      </c>
       <c r="G3" s="5">
         <v>1410071973</v>
       </c>
@@ -1154,6 +1189,9 @@
       <c r="D4" s="5" t="s">
         <v>37</v>
       </c>
+      <c r="F4" s="5">
+        <v>1410240211</v>
+      </c>
       <c r="G4" s="5">
         <v>1410240211</v>
       </c>
@@ -1241,6 +1279,9 @@
       <c r="D5" s="5" t="s">
         <v>37</v>
       </c>
+      <c r="F5" s="5">
+        <v>1917787990</v>
+      </c>
       <c r="G5" s="5">
         <v>1410436602</v>
       </c>
@@ -1328,6 +1369,9 @@
       <c r="D6" s="5" t="s">
         <v>37</v>
       </c>
+      <c r="F6" s="5">
+        <v>1305213723</v>
+      </c>
       <c r="G6" s="5">
         <v>1410213723</v>
       </c>
@@ -1415,6 +1459,9 @@
       <c r="D7" s="5" t="s">
         <v>37</v>
       </c>
+      <c r="F7" s="5">
+        <v>1990757830</v>
+      </c>
       <c r="G7" s="5">
         <v>1410173774</v>
       </c>
@@ -1624,7 +1671,9 @@
       <c r="P9" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="Q9" s="7"/>
+      <c r="Q9" s="7">
+        <v>1731580504974</v>
+      </c>
       <c r="R9" s="5" t="s">
         <v>58</v>
       </c>
@@ -1722,14 +1771,38 @@
       </c>
       <c r="Q10" s="7"/>
       <c r="S10" s="8"/>
+      <c r="T10" s="5" t="s">
+        <v>126</v>
+      </c>
       <c r="U10" s="5" t="s">
         <v>124</v>
       </c>
+      <c r="V10" s="5">
+        <v>1834674262</v>
+      </c>
       <c r="W10" s="5" t="s">
         <v>125</v>
       </c>
+      <c r="X10" s="5" t="s">
+        <v>127</v>
+      </c>
       <c r="Y10" s="5" t="s">
         <v>78</v>
+      </c>
+      <c r="Z10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA10" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="AB10" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC10" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="AD10" s="5" t="s">
+        <v>129</v>
       </c>
       <c r="AE10" s="5" t="s">
         <v>69</v>
@@ -1763,6 +1836,9 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="Q1:Q1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V1:V1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>